<commit_message>
Fix Amazon rising links
</commit_message>
<xml_diff>
--- a/us_small_product_demand_finder.xlsx
+++ b/us_small_product_demand_finder.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb4f011faf7e14aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Small Product Tracker" sheetId="2" r:id="Ra2efdd5f524846da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7-Day Workflow" sheetId="3" r:id="R4795614082f94b51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Outreach" sheetId="4" r:id="R328eee593e734ffc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing Test Brief" sheetId="5" r:id="R8ea62bc7de194e34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Compliance" sheetId="6" r:id="R5935303a426846af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid List" sheetId="7" r:id="R315b6b624ffc4e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7c8b6abc02724b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Small Product Tracker" sheetId="2" r:id="R69b0e7e462c14dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7-Day Workflow" sheetId="3" r:id="R8ab6563439fb485e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Outreach" sheetId="4" r:id="R757936ea6be74c71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing Test Brief" sheetId="5" r:id="R3a146808e09e49fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Compliance" sheetId="6" r:id="R909a411b31f048ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid List" sheetId="7" r:id="R1a1aab05a7fd474c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,7 +578,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddd50e06b56a488c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R216ec345960a46f6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1194,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5db2b47d246479e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5149f85d1b5d4242"/>
 </x:worksheet>
 </file>
 
@@ -4612,7 +4612,7 @@
         <x:v>Capture 50 small product ideas</x:v>
       </x:c>
       <x:c r="C4" s="43" t="str">
-        <x:v>AliExpress top selling/Choice, 1688 source, Amazon Movers &amp; Shakers, TikTok Creative Center, Google Trends US.</x:v>
+        <x:v>AliExpress top selling/Choice, 1688 source, Amazon Search plus category-specific Amazon Rising lists, TikTok Creative Center, Google Trends US.</x:v>
       </x:c>
       <x:c r="D4" s="44" t="str">
         <x:v>50 candidate rows with price, signals, complaint and upgrade angle.</x:v>
@@ -5056,16 +5056,16 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="45" t="str">
-        <x:v>Amazon Movers &amp; Shakers</x:v>
+        <x:v>Amazon category-specific Movers &amp; Shakers</x:v>
       </x:c>
       <x:c r="B6" s="46" t="str">
-        <x:v>Fastest sales-rank gainers</x:v>
+        <x:v>Fastest sales-rank gainers inside the matching category</x:v>
       </x:c>
       <x:c r="C6" s="46" t="str">
-        <x:v>See short-term US demand changes.</x:v>
+        <x:v>See short-term US demand changes without landing on personalized Books/series pages.</x:v>
       </x:c>
       <x:c r="D6" s="47" t="str">
-        <x:v>https://www.amazon.com/gp/movers-and-shakers</x:v>
+        <x:v>https://www.amazon.com/gp/movers-and-shakers/home-garden/</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>

<commit_message>
Use broad Google Trends keywords
</commit_message>
<xml_diff>
--- a/us_small_product_demand_finder.xlsx
+++ b/us_small_product_demand_finder.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R7c8b6abc02724b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Small Product Tracker" sheetId="2" r:id="R69b0e7e462c14dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7-Day Workflow" sheetId="3" r:id="R8ab6563439fb485e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Outreach" sheetId="4" r:id="R757936ea6be74c71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing Test Brief" sheetId="5" r:id="R3a146808e09e49fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Compliance" sheetId="6" r:id="R909a411b31f048ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid List" sheetId="7" r:id="R1a1aab05a7fd474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6a1c8855552c4e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="US Small Product Tracker" sheetId="2" r:id="R733fa2570bf34622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7-Day Workflow" sheetId="3" r:id="Rb806f5e600b040f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Outreach" sheetId="4" r:id="Rb0afb3ed67fe4b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Landing Test Brief" sheetId="5" r:id="Re8b70a4b1cfa4a10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Compliance" sheetId="6" r:id="R3e74a72c79b34a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Avoid List" sheetId="7" r:id="Rb054c12045b74c61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -578,7 +578,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R216ec345960a46f6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb16a366757b54195"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1194,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5149f85d1b5d4242"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c306386bbcd4a54"/>
 </x:worksheet>
 </file>
 
@@ -5087,13 +5087,13 @@
         <x:v>Google Trends</x:v>
       </x:c>
       <x:c r="B8" s="46" t="str">
-        <x:v>US region/time/category search interest</x:v>
+        <x:v>2-3 broad consumer keywords, not long SKU phrases</x:v>
       </x:c>
       <x:c r="C8" s="46" t="str">
-        <x:v>Check whether demand is rising or stable.</x:v>
+        <x:v>Check whether demand is rising or stable without getting no-data pages.</x:v>
       </x:c>
       <x:c r="D8" s="47" t="str">
-        <x:v>https://trends.google.com/trends/</x:v>
+        <x:v>https://trends.google.com/trends/explore?date=today%2012-m&amp;geo=US&amp;q=desk%20organizer,home%20office,desk%20setup</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>